<commit_message>
feat(tests): update frontend relief, inventory, and dark mode flows
</commit_message>
<xml_diff>
--- a/tests/sample-imports/inventory-goods-sample.xlsx
+++ b/tests/sample-imports/inventory-goods-sample.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="11580"/>
+    <workbookView windowWidth="28800" windowHeight="12180"/>
   </bookViews>
   <sheets>
     <sheet name="Goods Import" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>Item Name</t>
   </si>
@@ -44,7 +44,7 @@
     <t>Notes</t>
   </si>
   <si>
-    <t>expiry</t>
+    <t>Expiration Date</t>
   </si>
   <si>
     <t>Family Pack Rice</t>
@@ -57,18 +57,6 @@
   </si>
   <si>
     <t>Sample goods row for active Goods import.</t>
-  </si>
-  <si>
-    <t>Bottled Water</t>
-  </si>
-  <si>
-    <t>Drinks</t>
-  </si>
-  <si>
-    <t>cases</t>
-  </si>
-  <si>
-    <t>Second goods row.</t>
   </si>
 </sst>
 </file>
@@ -1118,34 +1106,17 @@
         <v>9</v>
       </c>
       <c r="I2" s="1">
-        <v>46183</v>
+        <v>46213</v>
       </c>
     </row>
     <row r="3" spans="1:9">
-      <c r="A3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3">
-        <v>80</v>
-      </c>
-      <c r="D3" t="s">
-        <v>12</v>
-      </c>
-      <c r="E3" t="s">
-        <v>13</v>
-      </c>
-      <c r="I3" s="1">
-        <v>46176</v>
-      </c>
+      <c r="I3" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
   <ignoredErrors>
-    <ignoredError sqref="A1:E3" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:E2" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>